<commit_message>
chore: atualiza planilha de custo de papel
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JETAPRINT_Planilha_Custo_Papel.xlsx
+++ b/JETAPRINT_Planilha_Custo_Papel.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JETA_PRINT\JetaFlow_Calculadora\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JETAPRINT\JetaFlow_Calculadora\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B90EB762-3969-4189-8498-F53786529D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E71E88-5438-40CD-8AE5-F423627B3121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4B197B12-5550-4599-97DF-3173620B9B72}"/>
   </bookViews>
@@ -44,15 +44,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
   <si>
-    <t>Papél</t>
-  </si>
-  <si>
     <t>marca</t>
   </si>
   <si>
-    <t>Gramatura</t>
-  </si>
-  <si>
     <t xml:space="preserve">Duplex </t>
   </si>
   <si>
@@ -65,9 +59,6 @@
     <t>Battaglia</t>
   </si>
   <si>
-    <t>medidas (cm)</t>
-  </si>
-  <si>
     <t>Sulfite</t>
   </si>
   <si>
@@ -80,9 +71,6 @@
     <t>Suzano</t>
   </si>
   <si>
-    <t>Resma Fls</t>
-  </si>
-  <si>
     <t>Couche brilho</t>
   </si>
   <si>
@@ -92,9 +80,6 @@
     <t>64x88</t>
   </si>
   <si>
-    <t>PREÇO</t>
-  </si>
-  <si>
     <t>Off-set</t>
   </si>
   <si>
@@ -135,6 +120,21 @@
   </si>
   <si>
     <t>CAC</t>
+  </si>
+  <si>
+    <t>Formato (cm)</t>
+  </si>
+  <si>
+    <t>Quantidade folhas por Resma</t>
+  </si>
+  <si>
+    <t>Tipo de Papél</t>
+  </si>
+  <si>
+    <t>Gramatura (g)</t>
+  </si>
+  <si>
+    <t>PREÇO P RESMA</t>
   </si>
 </sst>
 </file>
@@ -540,38 +540,38 @@
     <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="E2" s="1">
         <v>100</v>
@@ -582,16 +582,16 @@
     </row>
     <row r="3" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B3" s="1">
         <v>75</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E3" s="1">
         <v>5000</v>
@@ -602,16 +602,16 @@
     </row>
     <row r="4" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="E4" s="1">
         <v>2500</v>
@@ -622,16 +622,16 @@
     </row>
     <row r="5" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E5" s="1">
         <v>250</v>
@@ -642,16 +642,16 @@
     </row>
     <row r="6" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E6" s="1">
         <v>125</v>
@@ -662,16 +662,16 @@
     </row>
     <row r="7" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E7" s="1">
         <v>250</v>
@@ -682,16 +682,16 @@
     </row>
     <row r="8" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E8" s="1">
         <v>250</v>
@@ -702,16 +702,16 @@
     </row>
     <row r="9" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E9" s="1">
         <v>250</v>
@@ -722,16 +722,16 @@
     </row>
     <row r="10" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E10" s="1">
         <v>250</v>
@@ -742,16 +742,16 @@
     </row>
     <row r="11" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B11" s="1">
         <v>170</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E11" s="1">
         <v>250</v>
@@ -762,16 +762,16 @@
     </row>
     <row r="12" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E12" s="1">
         <v>100</v>

</xml_diff>